<commit_message>
[auto-snapshot] 2026-04-17 00:00 | onda-hompage | 25 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_hair/동구_미용실.xlsx
+++ b/naver-place-crawler/results_hair/동구_미용실.xlsx
@@ -422,7 +422,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -567,11 +567,7 @@
           <t>블루가이</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>red8276@naver.com</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
@@ -661,11 +657,7 @@
           <t>헤어코코</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>n_n_v_v@naver.com</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
@@ -845,11 +837,7 @@
           <t>그린헤어샵</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>yjd4843@naver.com</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
@@ -1029,11 +1017,7 @@
           <t>찌꼬뽀꼬</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ggiccoppocco@naver.com</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
@@ -1299,11 +1283,7 @@
           <t>그린미용실</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>govl733@naver.com</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
@@ -1659,11 +1639,7 @@
           <t>긋시아헤어 동인천역 본점</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>lovedarl2@naver.com</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
@@ -1937,11 +1913,7 @@
           <t>블루마린미용실</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>hairyuep@naver.com</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
@@ -2031,11 +2003,7 @@
           <t>디오헤어</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>dojin440@naver.com</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
@@ -2125,11 +2093,7 @@
           <t>송이미용실</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>alohasy0792@naver.com</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
@@ -2219,11 +2183,7 @@
           <t>카리스마</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>jackieyou@naver.com</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
@@ -2403,11 +2363,7 @@
           <t>준헤어아트</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>jie0105@naver.com</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -2669,11 +2625,7 @@
           <t>살롱드비아</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>tpfud1124@naver.com</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
@@ -2763,11 +2715,7 @@
           <t>정아미용실</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>bora4141@naver.com</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -2939,11 +2887,7 @@
           <t>보헤미안헤어</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>125_suu@naver.com</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
@@ -3397,11 +3341,7 @@
           <t>김영선헤어파라팜</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>hjstylemm@naver.com</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
@@ -3491,11 +3431,7 @@
           <t>한지수헤어스타</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>love444477@naver.com</t>
-        </is>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
@@ -3585,11 +3521,7 @@
           <t>달컴헤어</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>moonsb1206@naver.com</t>
-        </is>
-      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
@@ -3679,11 +3611,7 @@
           <t>퀸헤어</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>ouou1771@naver.com</t>
-        </is>
-      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -3859,11 +3787,7 @@
           <t>젠틀맨</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>dannykim2010@naver.com</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
@@ -4129,11 +4053,7 @@
           <t>은지헤어샵</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>south0429@naver.com</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
@@ -4223,11 +4143,7 @@
           <t>헤어5.5</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>tnrua34@naver.com</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
@@ -4317,11 +4233,7 @@
           <t>칼라헤어샵</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>color63676@naver.com</t>
-        </is>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
@@ -4501,11 +4413,7 @@
           <t>예쁜머리</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>propshop@naver.com</t>
-        </is>
-      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
@@ -4681,11 +4589,7 @@
           <t>장헤어샵</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>jjongs10@naver.com</t>
-        </is>
-      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
@@ -4861,11 +4765,7 @@
           <t>N.5 송현점</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>nabannnn@naver.com</t>
-        </is>
-      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
@@ -5041,11 +4941,7 @@
           <t>올뎃헤어</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>gashwoon@naver.com</t>
-        </is>
-      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
@@ -5135,11 +5031,7 @@
           <t>유나샵</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>yuna10110@naver.com</t>
-        </is>
-      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
@@ -5409,11 +5301,7 @@
           <t>홈헤어살롱</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>jiyea_junjin@naver.com</t>
-        </is>
-      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -5499,11 +5387,7 @@
           <t>착한미용실</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>slayfox@naver.com</t>
-        </is>
-      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -5675,11 +5559,7 @@
           <t>착한미용실</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>slayfox@naver.com</t>
-        </is>
-      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
@@ -5863,11 +5743,7 @@
           <t>헤어박스</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>kpackage@naver.com</t>
-        </is>
-      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
@@ -6047,11 +5923,7 @@
           <t>아델라 헤어</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>hkhj8083@naver.com</t>
-        </is>
-      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
@@ -6141,11 +6013,7 @@
           <t>머리만들기</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>greencoy79@naver.com</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
@@ -6235,11 +6103,7 @@
           <t>레지나헤어</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>zipyzigi2001@naver.com</t>
-        </is>
-      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
@@ -6329,11 +6193,7 @@
           <t>미카엘헤어</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>lhw2611@naver.com</t>
-        </is>
-      </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
@@ -6423,11 +6283,7 @@
           <t>남자만들기</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>timmy0326@naver.com</t>
-        </is>
-      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
@@ -6517,11 +6373,7 @@
           <t>임진선헤어모드</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>hjstylemm@naver.com</t>
-        </is>
-      </c>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
@@ -6611,11 +6463,7 @@
           <t>진헤어</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>sspmj501@naver.com</t>
-        </is>
-      </c>
+      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
@@ -6889,11 +6737,7 @@
           <t>아이원헤어</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>leeareum96@naver.com</t>
-        </is>
-      </c>
+      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
@@ -6983,11 +6827,7 @@
           <t>더끌림헤어</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>kklim7512820@naver.com</t>
-        </is>
-      </c>
+      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -7073,11 +6913,7 @@
           <t>젠틀맨</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>dannykim2010@naver.com</t>
-        </is>
-      </c>
+      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
@@ -7253,11 +7089,7 @@
           <t>현대이발관</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>sacheoncity@naver.com</t>
-        </is>
-      </c>
+      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -7343,11 +7175,7 @@
           <t>시대이발관</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>ic-museum@naver.com</t>
-        </is>
-      </c>
+      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-17 04:00 | onda-hompage | 31 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_hair/동구_미용실.xlsx
+++ b/naver-place-crawler/results_hair/동구_미용실.xlsx
@@ -422,7 +422,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -567,7 +567,11 @@
           <t>블루가이</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>duswls1338@naver.com</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
@@ -642,7 +646,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -657,7 +661,11 @@
           <t>헤어코코</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>n_n_v_v@naver.com</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
@@ -732,7 +740,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -747,7 +755,11 @@
           <t>헤어블리스</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mini2028@naver.com</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
@@ -822,7 +834,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -837,7 +849,11 @@
           <t>그린헤어샵</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>yjd4843@naver.com</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
@@ -912,7 +928,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -927,7 +943,11 @@
           <t>웨이비헤어</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>banana2728@naver.com</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
@@ -1002,7 +1022,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1037,11 @@
           <t>찌꼬뽀꼬</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ggiccoppocco@naver.com</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
@@ -1092,7 +1116,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1131,11 @@
           <t>신데렐라헤어살롱</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>wonjung8542@naver.com</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
@@ -1182,7 +1210,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1225,11 @@
           <t>다가즈 헤어 동인천점</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>tmxkdlf70@naver.com</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -1243,13 +1275,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="Q9" t="n">
         <v>4</v>
       </c>
       <c r="R9" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1268,7 +1300,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1315,11 @@
           <t>그린미용실</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>govl733@naver.com</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
@@ -1358,7 +1394,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1409,11 @@
           <t>고은헤어</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>goodkej104@naver.com</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -1444,7 +1484,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1499,11 @@
           <t>오르세헤어</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>dhgngkstlek@naver.com</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
@@ -1534,7 +1578,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1593,11 @@
           <t>헤어 림</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>amurug1_nuna@naver.com</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
@@ -1624,7 +1672,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1687,11 @@
           <t>긋시아헤어 동인천역 본점</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>lovedarl2@naver.com</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
@@ -1714,7 +1766,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1860,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1875,11 @@
           <t>요미살롱</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>minji_3-@naver.com</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
@@ -1898,7 +1954,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1969,11 @@
           <t>블루마린미용실</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>hairyuep@naver.com</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
@@ -1988,7 +2048,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2063,11 @@
           <t>디오헤어</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dojin440@naver.com</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
@@ -2078,7 +2142,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2157,11 @@
           <t>송이미용실</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>alohasy0792@naver.com</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
@@ -2168,7 +2236,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2251,11 @@
           <t>카리스마</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>jackieyou@naver.com</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
@@ -2258,7 +2330,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2345,11 @@
           <t>나타나엘헤어</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>yuujiin@naver.com</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
@@ -2348,7 +2424,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2439,11 @@
           <t>준헤어아트</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>jie0105@naver.com</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -2434,7 +2514,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2529,11 @@
           <t>에스제이헤어</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>emkim1003@naver.com</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -2520,7 +2604,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2619,11 @@
           <t>어나더스타일</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>jadenchoe@naver.com</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
@@ -2610,7 +2698,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2788,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2803,11 @@
           <t>정아미용실</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>bora4141@naver.com</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -2786,7 +2878,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2893,11 @@
           <t>태쁘헤어</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tjdwlsl2004@naver.com</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -2872,7 +2968,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2983,11 @@
           <t>보헤미안헤어</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>125_suu@naver.com</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
@@ -2962,7 +3062,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -2977,7 +3077,11 @@
           <t>양지헤어모디컬 송림1호점</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>justdoit0706@naver.com</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
@@ -3052,7 +3156,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3171,11 @@
           <t>조이헤어샵</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>wedbl@naver.com</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
@@ -3142,7 +3250,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3265,11 @@
           <t>솔빛헤어샾</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>lovesmoothz@naver.com</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
@@ -3232,7 +3344,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3438,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3453,11 @@
           <t>김영선헤어파라팜</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>hjstylemm@naver.com</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
@@ -3416,7 +3532,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3622,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3637,11 @@
           <t>달컴헤어</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>moonsb1206@naver.com</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
@@ -3596,7 +3716,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3731,11 @@
           <t>퀸헤어</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ouou1771@naver.com</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -3682,7 +3806,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3697,7 +3821,11 @@
           <t>아가페헤어모드</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>hiksanin@naver.com</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
@@ -3772,7 +3900,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3915,11 @@
           <t>젠틀맨</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>dannykim2010@naver.com</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
@@ -3862,7 +3994,7 @@
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3877,7 +4009,11 @@
           <t>루나헤어</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>hott0116@naver.com</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -3948,7 +4084,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3963,7 +4099,11 @@
           <t>앨리스헤어</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>oh-hair@naver.com</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
@@ -4038,7 +4178,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4268,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4283,11 @@
           <t>헤어5.5</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>tnrua34@naver.com</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
@@ -4218,7 +4362,7 @@
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4377,11 @@
           <t>칼라헤어샵</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>color63676@naver.com</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
@@ -4308,7 +4456,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4471,11 @@
           <t>오늘은머리하는날</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>uiryeonginfo@naver.com</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
@@ -4398,7 +4550,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4565,11 @@
           <t>예쁜머리</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>propshop@naver.com</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
@@ -4484,7 +4640,7 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4655,11 @@
           <t>그녀는예뻤다헤어샵</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>curablee@naver.com</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
@@ -4574,7 +4734,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4749,11 @@
           <t>장헤어샵</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>jjongs10@naver.com</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
@@ -4660,7 +4824,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4839,11 @@
           <t>모퉁이미장원</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>nijal99@naver.com</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
@@ -4750,7 +4918,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4933,11 @@
           <t>N.5 송현점</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>nabannnn@naver.com</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
@@ -4836,7 +5008,7 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4851,7 +5023,11 @@
           <t>챠밍헤어클럽</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>dongsimgi1004@naver.com</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
@@ -4926,7 +5102,7 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4941,7 +5117,11 @@
           <t>올뎃헤어</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>gashwoon@naver.com</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
@@ -5016,7 +5196,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5211,11 @@
           <t>유나샵</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>yuna10110@naver.com</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
@@ -5106,7 +5290,7 @@
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5305,11 @@
           <t>은헤어샵</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>dla_dp_fls@naver.com</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
@@ -5196,7 +5384,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5211,7 +5399,11 @@
           <t>장미미용실</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>shanyingstar@naver.com</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
@@ -5286,7 +5478,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5493,11 @@
           <t>홈헤어살롱</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>jiyea_junjin@naver.com</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -5372,7 +5568,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5583,11 @@
           <t>착한미용실</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>slayfox@naver.com</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -5458,7 +5658,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5744,7 @@
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5759,11 @@
           <t>착한미용실</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>slayfox@naver.com</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
@@ -5634,7 +5838,7 @@
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5932,7 @@
       </c>
       <c r="V59" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5947,11 @@
           <t>헤어박스</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>kpackage@naver.com</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
@@ -5818,7 +6026,7 @@
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5833,7 +6041,11 @@
           <t>초이스헤어</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>nrzzzzzz@naver.com</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
@@ -5908,7 +6120,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -5998,7 +6210,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6088,7 +6300,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6315,11 @@
           <t>레지나헤어</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>zipyzigi2001@naver.com</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
@@ -6178,7 +6394,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6409,11 @@
           <t>미카엘헤어</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>lhw2611@naver.com</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
@@ -6268,7 +6488,7 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6503,11 @@
           <t>남자만들기</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>timmy0326@naver.com</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
@@ -6358,7 +6582,7 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6597,11 @@
           <t>임진선헤어모드</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>hjstylemm@naver.com</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
@@ -6448,7 +6676,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6463,7 +6691,11 @@
           <t>진헤어</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>sspmj501@naver.com</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
@@ -6538,7 +6770,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6553,7 +6785,11 @@
           <t>꽃잎사이다</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>movie6miri@naver.com</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
@@ -6628,7 +6864,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6722,7 +6958,7 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6737,7 +6973,11 @@
           <t>아이원헤어</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>leeareum96@naver.com</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
@@ -6812,7 +7052,7 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6827,7 +7067,11 @@
           <t>더끌림헤어</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>kklim7512820@naver.com</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -6898,7 +7142,7 @@
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -6913,7 +7157,11 @@
           <t>젠틀맨</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>dannykim2010@naver.com</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
@@ -6988,7 +7236,7 @@
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7251,11 @@
           <t>서흥이발관</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>humble6551@naver.com</t>
+        </is>
+      </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
@@ -7074,7 +7326,7 @@
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7341,11 @@
           <t>현대이발관</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>sacheoncity@naver.com</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -7160,7 +7416,7 @@
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -7175,7 +7431,11 @@
           <t>시대이발관</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ic-museum@naver.com</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
@@ -7250,7 +7510,7 @@
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-17 08:00 | onda-hompage | 22 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_hair/동구_미용실.xlsx
+++ b/naver-place-crawler/results_hair/동구_미용실.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>duswls1338@naver.com</t>
+          <t>red8276@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -2713,7 +2713,11 @@
           <t>살롱드비아</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>tpfud1124@naver.com</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
@@ -3547,7 +3551,11 @@
           <t>한지수헤어스타</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>love444477@naver.com</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
@@ -3733,7 +3741,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ouou1771@naver.com</t>
+          <t>korea20027@naver.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -4193,7 +4201,11 @@
           <t>은지헤어샵</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>south0429@naver.com</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
@@ -5673,7 +5685,11 @@
           <t>다온헤어</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>gjraby00@naver.com</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -6135,7 +6151,11 @@
           <t>아델라 헤어</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>hkhj8083@naver.com</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
@@ -6225,7 +6245,11 @@
           <t>머리만들기</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>greencoy79@naver.com</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>

</xml_diff>